<commit_message>
Training example: ADS-B fuel flows consistent with power setting
fuel_flow (aircraft total) = 2 x ICAO fuel flow of 01P20CM128 at the
row's power setting (linear on the four ICAO points); PHRTM power below
idle raised to 0.07. Positions, altitude, TAS and times unchanged.
training_out and training_v3 studies patched; only bffm2_traj moves
(example NOx 17.4610 -> 18.7213 kg, movement 11); pinned CSV,
workbooks and docs regenerated. Sub-idle warning no longer fires on the
shipped example.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GmUEdC5zxhaEPVR7fnYi1y
</commit_message>
<xml_diff>
--- a/example/training/training_validation_reference.xlsx
+++ b/example/training/training_validation_reference.xlsx
@@ -490,7 +490,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Worst relative gap plugin vs reference: 2.4e-13 on the ANP movements, 4.4e-05 on movement 11 (CUSTOM profile, supplied track).</t>
+          <t>Worst relative gap plugin vs reference: 2.4e-13 on the ANP movements, 4.1e-06 on movement 11 (CUSTOM profile, supplied track).</t>
         </is>
       </c>
     </row>
@@ -745,10 +745,10 @@
         <v>22.41416778264804</v>
       </c>
       <c r="D3" t="n">
-        <v>23.65126116177226</v>
+        <v>23.33770314995289</v>
       </c>
       <c r="E3" t="n">
-        <v>23.65119517992509</v>
+        <v>23.33770300719163</v>
       </c>
       <c r="F3" t="n">
         <v>21.94877074704628</v>
@@ -776,10 +776,10 @@
         <v>7702.95181693998</v>
       </c>
       <c r="D4" t="n">
-        <v>6009.303801314025</v>
+        <v>6385.836677226731</v>
       </c>
       <c r="E4" t="n">
-        <v>6009.294901128162</v>
+        <v>6385.835011126059</v>
       </c>
       <c r="F4" t="n">
         <v>7708.835474860139</v>
@@ -807,10 +807,10 @@
         <v>1.227822241879149</v>
       </c>
       <c r="D5" t="n">
-        <v>1.2542543505182</v>
+        <v>1.252468181913424</v>
       </c>
       <c r="E5" t="n">
-        <v>1.254253465879471</v>
+        <v>1.252468170492528</v>
       </c>
       <c r="F5" t="n">
         <v>1.237476793718553</v>
@@ -838,10 +838,10 @@
         <v>31.84088970009263</v>
       </c>
       <c r="D6" t="n">
-        <v>17.4610078635899</v>
+        <v>18.72134446485447</v>
       </c>
       <c r="E6" t="n">
-        <v>17.46099724968429</v>
+        <v>18.7213383372177</v>
       </c>
       <c r="F6" t="n">
         <v>30.05600124882837</v>
@@ -869,10 +869,10 @@
         <v>1.848562177486793</v>
       </c>
       <c r="D7" t="n">
-        <v>1.442118811610278</v>
+        <v>1.532479552470924</v>
       </c>
       <c r="E7" t="n">
-        <v>1.442116675734661</v>
+        <v>1.532479152638397</v>
       </c>
       <c r="F7" t="n">
         <v>1.849974143672607</v>
@@ -900,10 +900,10 @@
         <v>0.3219805824842527</v>
       </c>
       <c r="D8" t="n">
-        <v>0.2854250095578111</v>
+        <v>0.2916112707090255</v>
       </c>
       <c r="E8" t="n">
-        <v>0.2854248639011709</v>
+        <v>0.291611243442336</v>
       </c>
       <c r="F8" t="n">
         <v>0.3222922906539849</v>
@@ -2551,10 +2551,10 @@
         <v>1.239981802111557</v>
       </c>
       <c r="E14" t="n">
-        <v>1.517123059722133</v>
+        <v>1.203565047902762</v>
       </c>
       <c r="F14" t="n">
-        <v>1.517057077875044</v>
+        <v>1.203564905141588</v>
       </c>
       <c r="G14" t="n">
         <v>1.229304479945856</v>
@@ -2569,10 +2569,10 @@
         <v>896.6548282456466</v>
       </c>
       <c r="K14" t="n">
-        <v>204.6423022099099</v>
+        <v>581.1751781226151</v>
       </c>
       <c r="L14" t="n">
-        <v>204.6334020241235</v>
+        <v>581.1735120220202</v>
       </c>
       <c r="M14" t="n">
         <v>881.5683619073927</v>
@@ -2587,10 +2587,10 @@
         <v>0.02041703055851676</v>
       </c>
       <c r="Q14" t="n">
-        <v>0.02034053108272857</v>
+        <v>0.01855436247795308</v>
       </c>
       <c r="R14" t="n">
-        <v>0.02033964644400199</v>
+        <v>0.01855435105705928</v>
       </c>
       <c r="S14" t="n">
         <v>0.02061351704140056</v>
@@ -2605,10 +2605,10 @@
         <v>3.836516818567063</v>
       </c>
       <c r="W14" t="n">
-        <v>0.2440459320356641</v>
+        <v>1.50438253330024</v>
       </c>
       <c r="X14" t="n">
-        <v>0.2440353181297802</v>
+        <v>1.504376405663195</v>
       </c>
       <c r="Y14" t="n">
         <v>4.109231807499004</v>
@@ -2623,10 +2623,10 @@
         <v>0.2151801336872796</v>
       </c>
       <c r="AC14" t="n">
-        <v>0.04911026691704524</v>
+        <v>0.1394710077776911</v>
       </c>
       <c r="AD14" t="n">
-        <v>0.04910813104144738</v>
+        <v>0.1394706079451831</v>
       </c>
       <c r="AE14" t="n">
         <v>0.2115596682179912</v>
@@ -2641,10 +2641,10 @@
         <v>0.01469376702111024</v>
       </c>
       <c r="AI14" t="n">
-        <v>0.003337385138824306</v>
+        <v>0.009523646290038726</v>
       </c>
       <c r="AJ14" t="n">
-        <v>0.003337239482182449</v>
+        <v>0.009523619023347505</v>
       </c>
       <c r="AK14" t="n">
         <v>0.01444821479277915</v>
@@ -2903,10 +2903,10 @@
         <v>22.41416778264804</v>
       </c>
       <c r="E17" t="n">
-        <v>23.65126116177226</v>
+        <v>23.33770314995289</v>
       </c>
       <c r="F17" t="n">
-        <v>23.65119517992509</v>
+        <v>23.33770300719163</v>
       </c>
       <c r="G17" t="n">
         <v>21.94877074704628</v>
@@ -2921,10 +2921,10 @@
         <v>7702.95181693998</v>
       </c>
       <c r="K17" t="n">
-        <v>6009.303801314025</v>
+        <v>6385.836677226731</v>
       </c>
       <c r="L17" t="n">
-        <v>6009.294901128162</v>
+        <v>6385.835011126059</v>
       </c>
       <c r="M17" t="n">
         <v>7708.835474860139</v>
@@ -2939,10 +2939,10 @@
         <v>1.227822241879149</v>
       </c>
       <c r="Q17" t="n">
-        <v>1.2542543505182</v>
+        <v>1.252468181913424</v>
       </c>
       <c r="R17" t="n">
-        <v>1.254253465879471</v>
+        <v>1.252468170492528</v>
       </c>
       <c r="S17" t="n">
         <v>1.237476793718553</v>
@@ -2957,10 +2957,10 @@
         <v>31.84088970009263</v>
       </c>
       <c r="W17" t="n">
-        <v>17.4610078635899</v>
+        <v>18.72134446485447</v>
       </c>
       <c r="X17" t="n">
-        <v>17.46099724968429</v>
+        <v>18.7213383372177</v>
       </c>
       <c r="Y17" t="n">
         <v>30.05600124882837</v>
@@ -2975,10 +2975,10 @@
         <v>1.848562177486793</v>
       </c>
       <c r="AC17" t="n">
-        <v>1.442118811610278</v>
+        <v>1.532479552470924</v>
       </c>
       <c r="AD17" t="n">
-        <v>1.442116675734661</v>
+        <v>1.532479152638397</v>
       </c>
       <c r="AE17" t="n">
         <v>1.849974143672607</v>
@@ -2993,10 +2993,10 @@
         <v>0.3219805824842527</v>
       </c>
       <c r="AI17" t="n">
-        <v>0.2854250095578111</v>
+        <v>0.2916112707090255</v>
       </c>
       <c r="AJ17" t="n">
-        <v>0.2854248639011709</v>
+        <v>0.291611243442336</v>
       </c>
       <c r="AK17" t="n">
         <v>0.3222922906539849</v>
@@ -3899,7 +3899,7 @@
         <v>3.650223216030941</v>
       </c>
       <c r="C9" t="n">
-        <v>3.956774968272925</v>
+        <v>3.643216956453553</v>
       </c>
       <c r="D9" t="n">
         <v>3.351670141385034</v>
@@ -3908,7 +3908,7 @@
         <v>1320.520166205253</v>
       </c>
       <c r="F9" t="n">
-        <v>571.2832888566306</v>
+        <v>947.8161647693357</v>
       </c>
       <c r="G9" t="n">
         <v>1291.724350092784</v>
@@ -3917,7 +3917,7 @@
         <v>0.2283253103540685</v>
       </c>
       <c r="I9" t="n">
-        <v>0.2301924480515556</v>
+        <v>0.2284062794467801</v>
       </c>
       <c r="J9" t="n">
         <v>0.2241571387179871</v>
@@ -3926,7 +3926,7 @@
         <v>4.69067743936141</v>
       </c>
       <c r="L9" t="n">
-        <v>0.8080439761362889</v>
+        <v>2.068380577400865</v>
       </c>
       <c r="M9" t="n">
         <v>4.824306176199871</v>
@@ -3935,7 +3935,7 @@
         <v>0.316899766721548</v>
       </c>
       <c r="O9" t="n">
-        <v>0.1370971421745371</v>
+        <v>0.2274578830351829</v>
       </c>
       <c r="P9" t="n">
         <v>0.3099893176105575</v>
@@ -3944,7 +3944,7 @@
         <v>0.03752844288525238</v>
       </c>
       <c r="R9" t="n">
-        <v>0.02503872770431084</v>
+        <v>0.03122498885552526</v>
       </c>
       <c r="S9" t="n">
         <v>0.03693974032739044</v>

</xml_diff>